<commit_message>
feat(reports): sablon chart bar renkleri + departman hucreleri center align
Sablon degisiklikleri (edit-template-charts-v2.js ile uygulandi):
 - frekansiyel-rapor-tumu.xlsx: chart2-chart9'a <c:dPt> elementleri
   eklendi. Her mini bar chart'ta 3 data point renkli:
     idx=0 (Hedef)      → 3B82F6 mavi
     idx=1 (Tamamlanan) → 10B981 yesil
     idx=2 (Sapma)      → F59E0B sari (amber)
 - frekansiyel-rapor-tek.xlsx: chart2-3 icin ayni (chart4-9 yok)

Backend endpoint:
 - Ozet row 17 (D17-AA17) departman hucrelerine
   alignment { horizontal: 'center', vertical: 'middle' } uygulandi.
   ExcelJS styles.xml'i overwrite ediyor -> sablon alignment kaybediyor,
   backend her hucreye tek tek set ediyor.

Sonuc: veriler ortali, chart bar'lari 3 renkli.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lib/reports/templates/frekansiyel-rapor-tumu.xlsx
+++ b/lib/reports/templates/frekansiyel-rapor-tumu.xlsx
@@ -3748,6 +3748,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$D$15:$F$16</c:f>
@@ -3995,6 +4037,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$G$15:$I$16</c:f>
@@ -4242,6 +4326,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$J$15:$L$16</c:f>
@@ -4489,6 +4615,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$M$15:$O$16</c:f>
@@ -4736,6 +4904,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$P$15:$R$16</c:f>
@@ -4983,6 +5193,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$S$15:$U$16</c:f>
@@ -5230,6 +5482,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$V$15:$X$16</c:f>
@@ -5477,6 +5771,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3B82F6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:multiLvlStrRef>
               <c:f>Özet!$Y$15:$AA$16</c:f>

</xml_diff>